<commit_message>
Update GitHub actions to mirror Appium & Selenium structures, inject CareerAI specific properties into Vulnerability framework
</commit_message>
<xml_diff>
--- a/vulnerability/automation/Vulnerability_Complete_Test_Report.xlsx
+++ b/vulnerability/automation/Vulnerability_Complete_Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2725" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2725" uniqueCount="369">
   <si>
     <t>Metric</t>
   </si>
@@ -68,10 +68,10 @@
     <t>SQL Injection (SQLi)</t>
   </si>
   <si>
-    <t>SQL Injection in User Login Email Field</t>
-  </si>
-  <si>
-    <t>/auth/verify-otp</t>
+    <t>SQL Injection in CareerAI Member Login Email Field</t>
+  </si>
+  <si>
+    <t>/api/auth/login-otp</t>
   </si>
   <si>
     <t>' OR 1=1; --</t>
@@ -95,10 +95,10 @@
     <t>Cross-Site Scripting (XSS)</t>
   </si>
   <si>
-    <t>Stored XSS in investigator full name parameter</t>
-  </si>
-  <si>
-    <t>/auth/request-otp</t>
+    <t>Stored XSS in Live Interviewer conversational parameter</t>
+  </si>
+  <si>
+    <t>/api/interviews/live</t>
   </si>
   <si>
     <t>&lt;script&gt;alert('xss')&lt;/script&gt;</t>
@@ -113,13 +113,13 @@
     <t>Command Injection / RCE</t>
   </si>
   <si>
-    <t>OS Command Injection via filename metadata header</t>
-  </si>
-  <si>
-    <t>/analyze-fast</t>
-  </si>
-  <si>
-    <t>sample_video.mp4; rm -rf /</t>
+    <t>OS Command Injection via Resume Analysis payload header</t>
+  </si>
+  <si>
+    <t>/api/resumes/analyze</t>
+  </si>
+  <si>
+    <t>resume_pdf.pdf; rm -rf /</t>
   </si>
   <si>
     <t>Strict path/filename sanitization; system strips special execution flags (';', '|', '&amp;').</t>
@@ -134,16 +134,16 @@
     <t>Path Traversal</t>
   </si>
   <si>
-    <t>Path Traversal payload in remote file downloader url</t>
-  </si>
-  <si>
-    <t>/analyze-pdf</t>
-  </si>
-  <si>
-    <t>https://safe-url.com/../../../../etc/passwd</t>
-  </si>
-  <si>
-    <t>Downloader checks path segments and restricts storage strictly to temp sandbox.</t>
+    <t>Path Traversal payload in Flashcard Deck exporter URL</t>
+  </si>
+  <si>
+    <t>/api/flashcards/export</t>
+  </si>
+  <si>
+    <t>https://careerai-system.com/../../../../etc/passwd</t>
+  </si>
+  <si>
+    <t>Exporter checks path segments and restricts storage strictly to CareerAI temp sandbox.</t>
   </si>
   <si>
     <t>A01:2021-Broken Access Control</t>
@@ -155,16 +155,16 @@
     <t>XML External Entity (XXE)</t>
   </si>
   <si>
-    <t>XXE injection in XML/SVG parser</t>
-  </si>
-  <si>
-    <t>/analyze-image</t>
+    <t>XXE injection in Job Application SVG/XML parser</t>
+  </si>
+  <si>
+    <t>/api/applications/upload</t>
   </si>
   <si>
     <t>&lt;!ENTITY xxe SYSTEM "file:///etc/passwd"&gt;</t>
   </si>
   <si>
-    <t>Deactivate resolution of external entity URIs in all image-parser libraries.</t>
+    <t>Deactivate resolution of external entity URIs in all CareerAI document-parser libraries.</t>
   </si>
   <si>
     <t>A05:2021-Security Misconfiguration</t>
@@ -176,10 +176,10 @@
     <t>Broken Authentication</t>
   </si>
   <si>
-    <t>Bypass login authentication by guessing active session token</t>
-  </si>
-  <si>
-    <t>/auth/check-session</t>
+    <t>Bypass login authentication by guessing active Mock Test token</t>
+  </si>
+  <si>
+    <t>/api/mock-tests/start</t>
   </si>
   <si>
     <t>Cookie: session_token=123</t>
@@ -197,16 +197,16 @@
     <t>Insecure CORS/CORS Misconfiguration</t>
   </si>
   <si>
-    <t>Access control origin headers set to wildcard '*' under authentication context</t>
-  </si>
-  <si>
-    <t>FastAPI Main configuration</t>
+    <t>Access control origin headers set to wildcard '*' under AI Engine context</t>
+  </si>
+  <si>
+    <t>CareerAI Engine Gateway</t>
   </si>
   <si>
     <t>Origin: http://attacker-domain.com</t>
   </si>
   <si>
-    <t>Allowed origins list strict configuration; wildcard deactivated on API.</t>
+    <t>Allowed origins list strict configuration; wildcard deactivated on AI APIs.</t>
   </si>
   <si>
     <t>TS_SEC_008</t>
@@ -215,10 +215,10 @@
     <t>Denial of Service (DoS/ReDoS)</t>
   </si>
   <si>
-    <t>Denial of Service via uploading zero-compression infinite frames archive</t>
-  </si>
-  <si>
-    <t>/analyze-video</t>
+    <t>Denial of Service via uploading zero-compression infinite Interview Video archive</t>
+  </si>
+  <si>
+    <t>/api/interviews/video-upload</t>
   </si>
   <si>
     <t>decompression_bomb.zip</t>
@@ -233,13 +233,16 @@
     <t>Malicious File Upload</t>
   </si>
   <si>
-    <t>Upload web shell payload renamed with video suffix</t>
-  </si>
-  <si>
-    <t>webshell.php.mp4</t>
-  </si>
-  <si>
-    <t>System validates mime type by actual bitstream signature, not extension.</t>
+    <t>Upload web shell payload renamed with Application Resume pdf suffix</t>
+  </si>
+  <si>
+    <t>/api/resumes/upload</t>
+  </si>
+  <si>
+    <t>webshell.php.pdf</t>
+  </si>
+  <si>
+    <t>CareerAI system validates mime type by actual bitstream signature, not extension.</t>
   </si>
   <si>
     <t>TS_SEC_010</t>
@@ -1818,13 +1821,13 @@
         <v>73</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G10" t="s">
         <v>22</v>
@@ -1838,7 +1841,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B11" t="s">
         <v>17</v>
@@ -1867,7 +1870,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
         <v>26</v>
@@ -1896,7 +1899,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
@@ -1925,7 +1928,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
         <v>39</v>
@@ -1954,7 +1957,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B15" t="s">
         <v>46</v>
@@ -1983,7 +1986,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
         <v>53</v>
@@ -2012,7 +2015,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
         <v>60</v>
@@ -2041,7 +2044,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B18" t="s">
         <v>66</v>
@@ -2070,7 +2073,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B19" t="s">
         <v>72</v>
@@ -2079,13 +2082,13 @@
         <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G19" t="s">
         <v>22</v>
@@ -2099,7 +2102,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
         <v>17</v>
@@ -2128,7 +2131,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" t="s">
         <v>26</v>
@@ -2157,7 +2160,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
         <v>32</v>
@@ -2186,7 +2189,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
         <v>39</v>
@@ -2215,7 +2218,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
         <v>46</v>
@@ -2244,7 +2247,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B25" t="s">
         <v>53</v>
@@ -2273,7 +2276,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B26" t="s">
         <v>60</v>
@@ -2302,7 +2305,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B27" t="s">
         <v>66</v>
@@ -2331,7 +2334,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B28" t="s">
         <v>72</v>
@@ -2340,13 +2343,13 @@
         <v>73</v>
       </c>
       <c r="D28" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E28" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G28" t="s">
         <v>22</v>
@@ -2360,7 +2363,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B29" t="s">
         <v>17</v>
@@ -2389,7 +2392,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B30" t="s">
         <v>26</v>
@@ -2418,7 +2421,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
@@ -2447,7 +2450,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B32" t="s">
         <v>39</v>
@@ -2476,7 +2479,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33" t="s">
         <v>46</v>
@@ -2505,7 +2508,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B34" t="s">
         <v>53</v>
@@ -2534,7 +2537,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B35" t="s">
         <v>60</v>
@@ -2563,7 +2566,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B36" t="s">
         <v>66</v>
@@ -2592,7 +2595,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B37" t="s">
         <v>72</v>
@@ -2601,13 +2604,13 @@
         <v>73</v>
       </c>
       <c r="D37" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G37" t="s">
         <v>22</v>
@@ -2621,7 +2624,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B38" t="s">
         <v>17</v>
@@ -2650,7 +2653,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B39" t="s">
         <v>26</v>
@@ -2679,7 +2682,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B40" t="s">
         <v>32</v>
@@ -2708,7 +2711,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B41" t="s">
         <v>39</v>
@@ -2737,7 +2740,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B42" t="s">
         <v>46</v>
@@ -2766,7 +2769,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B43" t="s">
         <v>53</v>
@@ -2795,7 +2798,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B44" t="s">
         <v>60</v>
@@ -2824,7 +2827,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B45" t="s">
         <v>66</v>
@@ -2853,7 +2856,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B46" t="s">
         <v>72</v>
@@ -2862,13 +2865,13 @@
         <v>73</v>
       </c>
       <c r="D46" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E46" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F46" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G46" t="s">
         <v>22</v>
@@ -2882,7 +2885,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B47" t="s">
         <v>17</v>
@@ -2911,7 +2914,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B48" t="s">
         <v>26</v>
@@ -2940,7 +2943,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B49" t="s">
         <v>32</v>
@@ -2969,7 +2972,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B50" t="s">
         <v>39</v>
@@ -2998,7 +3001,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B51" t="s">
         <v>46</v>
@@ -3027,7 +3030,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B52" t="s">
         <v>53</v>
@@ -3056,7 +3059,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B53" t="s">
         <v>60</v>
@@ -3085,7 +3088,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B54" t="s">
         <v>66</v>
@@ -3114,7 +3117,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B55" t="s">
         <v>72</v>
@@ -3123,13 +3126,13 @@
         <v>73</v>
       </c>
       <c r="D55" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E55" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F55" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G55" t="s">
         <v>22</v>
@@ -3143,7 +3146,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B56" t="s">
         <v>17</v>
@@ -3172,7 +3175,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B57" t="s">
         <v>26</v>
@@ -3201,7 +3204,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B58" t="s">
         <v>32</v>
@@ -3230,7 +3233,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B59" t="s">
         <v>39</v>
@@ -3259,7 +3262,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B60" t="s">
         <v>46</v>
@@ -3288,7 +3291,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B61" t="s">
         <v>53</v>
@@ -3317,7 +3320,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B62" t="s">
         <v>60</v>
@@ -3346,7 +3349,7 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B63" t="s">
         <v>66</v>
@@ -3375,7 +3378,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B64" t="s">
         <v>72</v>
@@ -3384,13 +3387,13 @@
         <v>73</v>
       </c>
       <c r="D64" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E64" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F64" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G64" t="s">
         <v>22</v>
@@ -3404,7 +3407,7 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B65" t="s">
         <v>17</v>
@@ -3433,7 +3436,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B66" t="s">
         <v>26</v>
@@ -3462,7 +3465,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B67" t="s">
         <v>32</v>
@@ -3491,7 +3494,7 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B68" t="s">
         <v>39</v>
@@ -3520,7 +3523,7 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B69" t="s">
         <v>46</v>
@@ -3549,7 +3552,7 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B70" t="s">
         <v>53</v>
@@ -3578,7 +3581,7 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B71" t="s">
         <v>60</v>
@@ -3607,7 +3610,7 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B72" t="s">
         <v>66</v>
@@ -3636,7 +3639,7 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B73" t="s">
         <v>72</v>
@@ -3645,13 +3648,13 @@
         <v>73</v>
       </c>
       <c r="D73" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E73" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F73" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G73" t="s">
         <v>22</v>
@@ -3665,7 +3668,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B74" t="s">
         <v>17</v>
@@ -3694,7 +3697,7 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B75" t="s">
         <v>26</v>
@@ -3723,7 +3726,7 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B76" t="s">
         <v>32</v>
@@ -3752,7 +3755,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B77" t="s">
         <v>39</v>
@@ -3781,7 +3784,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B78" t="s">
         <v>46</v>
@@ -3810,7 +3813,7 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B79" t="s">
         <v>53</v>
@@ -3839,7 +3842,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B80" t="s">
         <v>60</v>
@@ -3868,7 +3871,7 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B81" t="s">
         <v>66</v>
@@ -3897,7 +3900,7 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B82" t="s">
         <v>72</v>
@@ -3906,13 +3909,13 @@
         <v>73</v>
       </c>
       <c r="D82" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E82" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F82" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G82" t="s">
         <v>22</v>
@@ -3926,7 +3929,7 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B83" t="s">
         <v>17</v>
@@ -3955,7 +3958,7 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B84" t="s">
         <v>26</v>
@@ -3984,7 +3987,7 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B85" t="s">
         <v>32</v>
@@ -4013,7 +4016,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B86" t="s">
         <v>39</v>
@@ -4042,7 +4045,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B87" t="s">
         <v>46</v>
@@ -4071,7 +4074,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B88" t="s">
         <v>53</v>
@@ -4100,7 +4103,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B89" t="s">
         <v>60</v>
@@ -4129,7 +4132,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B90" t="s">
         <v>66</v>
@@ -4158,7 +4161,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B91" t="s">
         <v>72</v>
@@ -4167,13 +4170,13 @@
         <v>73</v>
       </c>
       <c r="D91" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E91" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F91" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G91" t="s">
         <v>22</v>
@@ -4187,7 +4190,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B92" t="s">
         <v>17</v>
@@ -4216,7 +4219,7 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B93" t="s">
         <v>26</v>
@@ -4245,7 +4248,7 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B94" t="s">
         <v>32</v>
@@ -4274,7 +4277,7 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B95" t="s">
         <v>39</v>
@@ -4303,7 +4306,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B96" t="s">
         <v>46</v>
@@ -4332,7 +4335,7 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B97" t="s">
         <v>53</v>
@@ -4361,7 +4364,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B98" t="s">
         <v>60</v>
@@ -4390,7 +4393,7 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B99" t="s">
         <v>66</v>
@@ -4419,7 +4422,7 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B100" t="s">
         <v>72</v>
@@ -4428,13 +4431,13 @@
         <v>73</v>
       </c>
       <c r="D100" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E100" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F100" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G100" t="s">
         <v>22</v>
@@ -4448,7 +4451,7 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B101" t="s">
         <v>17</v>
@@ -4477,7 +4480,7 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B102" t="s">
         <v>26</v>
@@ -4506,7 +4509,7 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B103" t="s">
         <v>32</v>
@@ -4535,7 +4538,7 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B104" t="s">
         <v>39</v>
@@ -4564,7 +4567,7 @@
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B105" t="s">
         <v>46</v>
@@ -4593,7 +4596,7 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B106" t="s">
         <v>53</v>
@@ -4622,7 +4625,7 @@
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B107" t="s">
         <v>60</v>
@@ -4651,7 +4654,7 @@
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B108" t="s">
         <v>66</v>
@@ -4680,7 +4683,7 @@
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B109" t="s">
         <v>72</v>
@@ -4689,13 +4692,13 @@
         <v>73</v>
       </c>
       <c r="D109" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E109" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F109" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G109" t="s">
         <v>22</v>
@@ -4709,7 +4712,7 @@
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B110" t="s">
         <v>17</v>
@@ -4738,7 +4741,7 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B111" t="s">
         <v>26</v>
@@ -4767,7 +4770,7 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B112" t="s">
         <v>32</v>
@@ -4796,7 +4799,7 @@
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B113" t="s">
         <v>39</v>
@@ -4825,7 +4828,7 @@
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B114" t="s">
         <v>46</v>
@@ -4854,7 +4857,7 @@
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B115" t="s">
         <v>53</v>
@@ -4883,7 +4886,7 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B116" t="s">
         <v>60</v>
@@ -4912,7 +4915,7 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B117" t="s">
         <v>66</v>
@@ -4941,7 +4944,7 @@
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B118" t="s">
         <v>72</v>
@@ -4950,13 +4953,13 @@
         <v>73</v>
       </c>
       <c r="D118" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E118" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F118" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G118" t="s">
         <v>22</v>
@@ -4970,7 +4973,7 @@
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B119" t="s">
         <v>17</v>
@@ -4999,7 +5002,7 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B120" t="s">
         <v>26</v>
@@ -5028,7 +5031,7 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B121" t="s">
         <v>32</v>
@@ -5057,7 +5060,7 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B122" t="s">
         <v>39</v>
@@ -5086,7 +5089,7 @@
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B123" t="s">
         <v>46</v>
@@ -5115,7 +5118,7 @@
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B124" t="s">
         <v>53</v>
@@ -5144,7 +5147,7 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B125" t="s">
         <v>60</v>
@@ -5173,7 +5176,7 @@
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B126" t="s">
         <v>66</v>
@@ -5202,7 +5205,7 @@
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B127" t="s">
         <v>72</v>
@@ -5211,13 +5214,13 @@
         <v>73</v>
       </c>
       <c r="D127" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E127" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F127" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G127" t="s">
         <v>22</v>
@@ -5231,7 +5234,7 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B128" t="s">
         <v>17</v>
@@ -5260,7 +5263,7 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B129" t="s">
         <v>26</v>
@@ -5289,7 +5292,7 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B130" t="s">
         <v>32</v>
@@ -5318,7 +5321,7 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B131" t="s">
         <v>39</v>
@@ -5347,7 +5350,7 @@
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B132" t="s">
         <v>46</v>
@@ -5376,7 +5379,7 @@
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B133" t="s">
         <v>53</v>
@@ -5405,7 +5408,7 @@
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B134" t="s">
         <v>60</v>
@@ -5434,7 +5437,7 @@
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B135" t="s">
         <v>66</v>
@@ -5463,7 +5466,7 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B136" t="s">
         <v>72</v>
@@ -5472,13 +5475,13 @@
         <v>73</v>
       </c>
       <c r="D136" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E136" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F136" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G136" t="s">
         <v>22</v>
@@ -5492,7 +5495,7 @@
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B137" t="s">
         <v>17</v>
@@ -5521,7 +5524,7 @@
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B138" t="s">
         <v>26</v>
@@ -5550,7 +5553,7 @@
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B139" t="s">
         <v>32</v>
@@ -5579,7 +5582,7 @@
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B140" t="s">
         <v>39</v>
@@ -5608,7 +5611,7 @@
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B141" t="s">
         <v>46</v>
@@ -5637,7 +5640,7 @@
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B142" t="s">
         <v>53</v>
@@ -5666,7 +5669,7 @@
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B143" t="s">
         <v>60</v>
@@ -5695,7 +5698,7 @@
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B144" t="s">
         <v>66</v>
@@ -5724,7 +5727,7 @@
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B145" t="s">
         <v>72</v>
@@ -5733,13 +5736,13 @@
         <v>73</v>
       </c>
       <c r="D145" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E145" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F145" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G145" t="s">
         <v>22</v>
@@ -5753,7 +5756,7 @@
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B146" t="s">
         <v>17</v>
@@ -5782,7 +5785,7 @@
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B147" t="s">
         <v>26</v>
@@ -5811,7 +5814,7 @@
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B148" t="s">
         <v>32</v>
@@ -5840,7 +5843,7 @@
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B149" t="s">
         <v>39</v>
@@ -5869,7 +5872,7 @@
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B150" t="s">
         <v>46</v>
@@ -5898,7 +5901,7 @@
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B151" t="s">
         <v>53</v>
@@ -5927,7 +5930,7 @@
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B152" t="s">
         <v>60</v>
@@ -5956,7 +5959,7 @@
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B153" t="s">
         <v>66</v>
@@ -5985,7 +5988,7 @@
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B154" t="s">
         <v>72</v>
@@ -5994,13 +5997,13 @@
         <v>73</v>
       </c>
       <c r="D154" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E154" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F154" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G154" t="s">
         <v>22</v>
@@ -6014,7 +6017,7 @@
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B155" t="s">
         <v>17</v>
@@ -6043,7 +6046,7 @@
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B156" t="s">
         <v>26</v>
@@ -6072,7 +6075,7 @@
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B157" t="s">
         <v>32</v>
@@ -6101,7 +6104,7 @@
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B158" t="s">
         <v>39</v>
@@ -6130,7 +6133,7 @@
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B159" t="s">
         <v>46</v>
@@ -6159,7 +6162,7 @@
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B160" t="s">
         <v>53</v>
@@ -6188,7 +6191,7 @@
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B161" t="s">
         <v>60</v>
@@ -6217,7 +6220,7 @@
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B162" t="s">
         <v>66</v>
@@ -6246,7 +6249,7 @@
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B163" t="s">
         <v>72</v>
@@ -6255,13 +6258,13 @@
         <v>73</v>
       </c>
       <c r="D163" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E163" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F163" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G163" t="s">
         <v>22</v>
@@ -6275,7 +6278,7 @@
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B164" t="s">
         <v>17</v>
@@ -6304,7 +6307,7 @@
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B165" t="s">
         <v>26</v>
@@ -6333,7 +6336,7 @@
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B166" t="s">
         <v>32</v>
@@ -6362,7 +6365,7 @@
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B167" t="s">
         <v>39</v>
@@ -6391,7 +6394,7 @@
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B168" t="s">
         <v>46</v>
@@ -6420,7 +6423,7 @@
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B169" t="s">
         <v>53</v>
@@ -6449,7 +6452,7 @@
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B170" t="s">
         <v>60</v>
@@ -6478,7 +6481,7 @@
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B171" t="s">
         <v>66</v>
@@ -6507,7 +6510,7 @@
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B172" t="s">
         <v>72</v>
@@ -6516,13 +6519,13 @@
         <v>73</v>
       </c>
       <c r="D172" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E172" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F172" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G172" t="s">
         <v>22</v>
@@ -6536,7 +6539,7 @@
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B173" t="s">
         <v>17</v>
@@ -6565,7 +6568,7 @@
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B174" t="s">
         <v>26</v>
@@ -6594,7 +6597,7 @@
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B175" t="s">
         <v>32</v>
@@ -6623,7 +6626,7 @@
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B176" t="s">
         <v>39</v>
@@ -6652,7 +6655,7 @@
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B177" t="s">
         <v>46</v>
@@ -6681,7 +6684,7 @@
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B178" t="s">
         <v>53</v>
@@ -6710,7 +6713,7 @@
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B179" t="s">
         <v>60</v>
@@ -6739,7 +6742,7 @@
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B180" t="s">
         <v>66</v>
@@ -6768,7 +6771,7 @@
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B181" t="s">
         <v>72</v>
@@ -6777,13 +6780,13 @@
         <v>73</v>
       </c>
       <c r="D181" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E181" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F181" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G181" t="s">
         <v>22</v>
@@ -6797,7 +6800,7 @@
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B182" t="s">
         <v>17</v>
@@ -6826,7 +6829,7 @@
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B183" t="s">
         <v>26</v>
@@ -6855,7 +6858,7 @@
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B184" t="s">
         <v>32</v>
@@ -6884,7 +6887,7 @@
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B185" t="s">
         <v>39</v>
@@ -6913,7 +6916,7 @@
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B186" t="s">
         <v>46</v>
@@ -6942,7 +6945,7 @@
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B187" t="s">
         <v>53</v>
@@ -6971,7 +6974,7 @@
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B188" t="s">
         <v>60</v>
@@ -7000,7 +7003,7 @@
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B189" t="s">
         <v>66</v>
@@ -7029,7 +7032,7 @@
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B190" t="s">
         <v>72</v>
@@ -7038,13 +7041,13 @@
         <v>73</v>
       </c>
       <c r="D190" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E190" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F190" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G190" t="s">
         <v>22</v>
@@ -7058,7 +7061,7 @@
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B191" t="s">
         <v>17</v>
@@ -7087,7 +7090,7 @@
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B192" t="s">
         <v>26</v>
@@ -7116,7 +7119,7 @@
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B193" t="s">
         <v>32</v>
@@ -7145,7 +7148,7 @@
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B194" t="s">
         <v>39</v>
@@ -7174,7 +7177,7 @@
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B195" t="s">
         <v>46</v>
@@ -7203,7 +7206,7 @@
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B196" t="s">
         <v>53</v>
@@ -7232,7 +7235,7 @@
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B197" t="s">
         <v>60</v>
@@ -7261,7 +7264,7 @@
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B198" t="s">
         <v>66</v>
@@ -7290,7 +7293,7 @@
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B199" t="s">
         <v>72</v>
@@ -7299,13 +7302,13 @@
         <v>73</v>
       </c>
       <c r="D199" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E199" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F199" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G199" t="s">
         <v>22</v>
@@ -7319,7 +7322,7 @@
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B200" t="s">
         <v>17</v>
@@ -7348,7 +7351,7 @@
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B201" t="s">
         <v>26</v>
@@ -7377,7 +7380,7 @@
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B202" t="s">
         <v>32</v>
@@ -7406,7 +7409,7 @@
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B203" t="s">
         <v>39</v>
@@ -7435,7 +7438,7 @@
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B204" t="s">
         <v>46</v>
@@ -7464,7 +7467,7 @@
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B205" t="s">
         <v>53</v>
@@ -7493,7 +7496,7 @@
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B206" t="s">
         <v>60</v>
@@ -7522,7 +7525,7 @@
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B207" t="s">
         <v>66</v>
@@ -7551,7 +7554,7 @@
     </row>
     <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B208" t="s">
         <v>72</v>
@@ -7560,13 +7563,13 @@
         <v>73</v>
       </c>
       <c r="D208" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E208" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F208" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G208" t="s">
         <v>22</v>
@@ -7580,7 +7583,7 @@
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B209" t="s">
         <v>17</v>
@@ -7609,7 +7612,7 @@
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B210" t="s">
         <v>26</v>
@@ -7638,7 +7641,7 @@
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B211" t="s">
         <v>32</v>
@@ -7667,7 +7670,7 @@
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B212" t="s">
         <v>39</v>
@@ -7696,7 +7699,7 @@
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B213" t="s">
         <v>46</v>
@@ -7725,7 +7728,7 @@
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B214" t="s">
         <v>53</v>
@@ -7754,7 +7757,7 @@
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B215" t="s">
         <v>60</v>
@@ -7783,7 +7786,7 @@
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B216" t="s">
         <v>66</v>
@@ -7812,7 +7815,7 @@
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B217" t="s">
         <v>72</v>
@@ -7821,13 +7824,13 @@
         <v>73</v>
       </c>
       <c r="D217" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E217" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F217" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G217" t="s">
         <v>22</v>
@@ -7841,7 +7844,7 @@
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B218" t="s">
         <v>17</v>
@@ -7870,7 +7873,7 @@
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B219" t="s">
         <v>26</v>
@@ -7899,7 +7902,7 @@
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B220" t="s">
         <v>32</v>
@@ -7928,7 +7931,7 @@
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B221" t="s">
         <v>39</v>
@@ -7957,7 +7960,7 @@
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B222" t="s">
         <v>46</v>
@@ -7986,7 +7989,7 @@
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B223" t="s">
         <v>53</v>
@@ -8015,7 +8018,7 @@
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B224" t="s">
         <v>60</v>
@@ -8044,7 +8047,7 @@
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B225" t="s">
         <v>66</v>
@@ -8073,7 +8076,7 @@
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B226" t="s">
         <v>72</v>
@@ -8082,13 +8085,13 @@
         <v>73</v>
       </c>
       <c r="D226" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E226" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F226" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G226" t="s">
         <v>22</v>
@@ -8102,7 +8105,7 @@
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B227" t="s">
         <v>17</v>
@@ -8131,7 +8134,7 @@
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B228" t="s">
         <v>26</v>
@@ -8160,7 +8163,7 @@
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B229" t="s">
         <v>32</v>
@@ -8189,7 +8192,7 @@
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B230" t="s">
         <v>39</v>
@@ -8218,7 +8221,7 @@
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B231" t="s">
         <v>46</v>
@@ -8247,7 +8250,7 @@
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B232" t="s">
         <v>53</v>
@@ -8276,7 +8279,7 @@
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B233" t="s">
         <v>60</v>
@@ -8305,7 +8308,7 @@
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B234" t="s">
         <v>66</v>
@@ -8334,7 +8337,7 @@
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B235" t="s">
         <v>72</v>
@@ -8343,13 +8346,13 @@
         <v>73</v>
       </c>
       <c r="D235" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E235" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F235" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G235" t="s">
         <v>22</v>
@@ -8363,7 +8366,7 @@
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B236" t="s">
         <v>17</v>
@@ -8392,7 +8395,7 @@
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B237" t="s">
         <v>26</v>
@@ -8421,7 +8424,7 @@
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B238" t="s">
         <v>32</v>
@@ -8450,7 +8453,7 @@
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B239" t="s">
         <v>39</v>
@@ -8479,7 +8482,7 @@
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B240" t="s">
         <v>46</v>
@@ -8508,7 +8511,7 @@
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B241" t="s">
         <v>53</v>
@@ -8537,7 +8540,7 @@
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B242" t="s">
         <v>60</v>
@@ -8566,7 +8569,7 @@
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B243" t="s">
         <v>66</v>
@@ -8595,7 +8598,7 @@
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B244" t="s">
         <v>72</v>
@@ -8604,13 +8607,13 @@
         <v>73</v>
       </c>
       <c r="D244" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E244" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F244" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G244" t="s">
         <v>22</v>
@@ -8624,7 +8627,7 @@
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B245" t="s">
         <v>17</v>
@@ -8653,7 +8656,7 @@
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B246" t="s">
         <v>26</v>
@@ -8682,7 +8685,7 @@
     </row>
     <row r="247" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B247" t="s">
         <v>32</v>
@@ -8711,7 +8714,7 @@
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B248" t="s">
         <v>39</v>
@@ -8740,7 +8743,7 @@
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B249" t="s">
         <v>46</v>
@@ -8769,7 +8772,7 @@
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B250" t="s">
         <v>53</v>
@@ -8798,7 +8801,7 @@
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B251" t="s">
         <v>60</v>
@@ -8827,7 +8830,7 @@
     </row>
     <row r="252" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B252" t="s">
         <v>66</v>
@@ -8856,7 +8859,7 @@
     </row>
     <row r="253" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B253" t="s">
         <v>72</v>
@@ -8865,13 +8868,13 @@
         <v>73</v>
       </c>
       <c r="D253" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E253" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F253" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G253" t="s">
         <v>22</v>
@@ -8885,7 +8888,7 @@
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B254" t="s">
         <v>17</v>
@@ -8914,7 +8917,7 @@
     </row>
     <row r="255" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B255" t="s">
         <v>26</v>
@@ -8943,7 +8946,7 @@
     </row>
     <row r="256" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B256" t="s">
         <v>32</v>
@@ -8972,7 +8975,7 @@
     </row>
     <row r="257" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B257" t="s">
         <v>39</v>
@@ -9001,7 +9004,7 @@
     </row>
     <row r="258" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B258" t="s">
         <v>46</v>
@@ -9030,7 +9033,7 @@
     </row>
     <row r="259" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B259" t="s">
         <v>53</v>
@@ -9059,7 +9062,7 @@
     </row>
     <row r="260" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B260" t="s">
         <v>60</v>
@@ -9088,7 +9091,7 @@
     </row>
     <row r="261" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B261" t="s">
         <v>66</v>
@@ -9117,7 +9120,7 @@
     </row>
     <row r="262" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B262" t="s">
         <v>72</v>
@@ -9126,13 +9129,13 @@
         <v>73</v>
       </c>
       <c r="D262" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E262" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F262" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G262" t="s">
         <v>22</v>
@@ -9146,7 +9149,7 @@
     </row>
     <row r="263" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B263" t="s">
         <v>17</v>
@@ -9175,7 +9178,7 @@
     </row>
     <row r="264" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B264" t="s">
         <v>26</v>
@@ -9204,7 +9207,7 @@
     </row>
     <row r="265" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B265" t="s">
         <v>32</v>
@@ -9233,7 +9236,7 @@
     </row>
     <row r="266" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B266" t="s">
         <v>39</v>
@@ -9262,7 +9265,7 @@
     </row>
     <row r="267" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B267" t="s">
         <v>46</v>
@@ -9291,7 +9294,7 @@
     </row>
     <row r="268" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B268" t="s">
         <v>53</v>
@@ -9320,7 +9323,7 @@
     </row>
     <row r="269" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B269" t="s">
         <v>60</v>
@@ -9349,7 +9352,7 @@
     </row>
     <row r="270" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B270" t="s">
         <v>66</v>
@@ -9378,7 +9381,7 @@
     </row>
     <row r="271" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B271" t="s">
         <v>72</v>
@@ -9387,13 +9390,13 @@
         <v>73</v>
       </c>
       <c r="D271" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E271" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F271" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G271" t="s">
         <v>22</v>
@@ -9407,7 +9410,7 @@
     </row>
     <row r="272" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B272" t="s">
         <v>17</v>
@@ -9436,7 +9439,7 @@
     </row>
     <row r="273" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B273" t="s">
         <v>26</v>
@@ -9465,7 +9468,7 @@
     </row>
     <row r="274" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B274" t="s">
         <v>32</v>
@@ -9494,7 +9497,7 @@
     </row>
     <row r="275" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B275" t="s">
         <v>39</v>
@@ -9523,7 +9526,7 @@
     </row>
     <row r="276" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B276" t="s">
         <v>46</v>
@@ -9552,7 +9555,7 @@
     </row>
     <row r="277" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B277" t="s">
         <v>53</v>
@@ -9581,7 +9584,7 @@
     </row>
     <row r="278" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B278" t="s">
         <v>60</v>
@@ -9610,7 +9613,7 @@
     </row>
     <row r="279" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B279" t="s">
         <v>66</v>
@@ -9639,7 +9642,7 @@
     </row>
     <row r="280" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B280" t="s">
         <v>72</v>
@@ -9648,13 +9651,13 @@
         <v>73</v>
       </c>
       <c r="D280" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E280" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F280" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G280" t="s">
         <v>22</v>
@@ -9668,7 +9671,7 @@
     </row>
     <row r="281" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B281" t="s">
         <v>17</v>
@@ -9697,7 +9700,7 @@
     </row>
     <row r="282" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B282" t="s">
         <v>26</v>
@@ -9726,7 +9729,7 @@
     </row>
     <row r="283" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B283" t="s">
         <v>32</v>
@@ -9755,7 +9758,7 @@
     </row>
     <row r="284" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B284" t="s">
         <v>39</v>
@@ -9784,7 +9787,7 @@
     </row>
     <row r="285" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B285" t="s">
         <v>46</v>
@@ -9813,7 +9816,7 @@
     </row>
     <row r="286" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B286" t="s">
         <v>53</v>
@@ -9842,7 +9845,7 @@
     </row>
     <row r="287" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B287" t="s">
         <v>60</v>
@@ -9871,7 +9874,7 @@
     </row>
     <row r="288" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B288" t="s">
         <v>66</v>
@@ -9900,7 +9903,7 @@
     </row>
     <row r="289" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B289" t="s">
         <v>72</v>
@@ -9909,13 +9912,13 @@
         <v>73</v>
       </c>
       <c r="D289" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E289" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F289" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G289" t="s">
         <v>22</v>
@@ -9929,7 +9932,7 @@
     </row>
     <row r="290" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B290" t="s">
         <v>17</v>
@@ -9958,7 +9961,7 @@
     </row>
     <row r="291" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B291" t="s">
         <v>26</v>
@@ -9987,7 +9990,7 @@
     </row>
     <row r="292" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B292" t="s">
         <v>32</v>
@@ -10016,7 +10019,7 @@
     </row>
     <row r="293" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B293" t="s">
         <v>39</v>
@@ -10045,7 +10048,7 @@
     </row>
     <row r="294" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B294" t="s">
         <v>46</v>
@@ -10074,7 +10077,7 @@
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B295" t="s">
         <v>53</v>
@@ -10103,7 +10106,7 @@
     </row>
     <row r="296" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B296" t="s">
         <v>60</v>
@@ -10132,7 +10135,7 @@
     </row>
     <row r="297" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B297" t="s">
         <v>66</v>
@@ -10161,7 +10164,7 @@
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B298" t="s">
         <v>72</v>
@@ -10170,13 +10173,13 @@
         <v>73</v>
       </c>
       <c r="D298" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E298" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F298" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G298" t="s">
         <v>22</v>
@@ -10190,7 +10193,7 @@
     </row>
     <row r="299" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B299" t="s">
         <v>17</v>
@@ -10219,7 +10222,7 @@
     </row>
     <row r="300" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B300" t="s">
         <v>26</v>
@@ -10248,7 +10251,7 @@
     </row>
     <row r="301" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B301" t="s">
         <v>32</v>
@@ -10277,7 +10280,7 @@
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B302" t="s">
         <v>39</v>

</xml_diff>